<commit_message>
RSL: 11 textos completos de ScienceDirect (42 extraídos, 37 en la síntesis)
- Lote 08: Li 2018, NFRNet, BERT-CNN, BERT-BiCNN, Casillo, Ali, Alsanoosy,
  Petrillo, Nguyen Van, Kaur 2026 y RequiBERT
- Dos estudios más remuestrean o aumentan antes de partir el conjunto (fuga)
- Resultados PR1, PR2, PR4 y PR5 actualizados; índice y formulario regenerados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Articulos/PDF/INDICE_ARTICULOS.xlsx
+++ b/Articulos/PDF/INDICE_ARTICULOS.xlsx
@@ -39,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -54,11 +54,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -89,15 +84,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -669,22 +663,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>06_ml_dl_clasico/9_Li2018_AutomaticallyClassifyingUserRequests.pdf</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>ML clásico</t>
@@ -1382,7 +1376,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -1476,22 +1470,22 @@
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>04_bert_transformers/71_Li2022_AutomaticallyClassifyingFunctionalRequir.pdf</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -1523,22 +1517,22 @@
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>04_bert_transformers/72_Kaur2022_BertImprovingBertRequirements.pdf</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -1621,7 +1615,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -1809,7 +1803,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -1903,7 +1897,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2001,7 +1995,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2052,7 +2046,7 @@
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -2095,7 +2089,7 @@
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2142,22 +2136,22 @@
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>04_bert_transformers/118_Kaur2023_ImprovingBertModelRequirements.pdf</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -2283,7 +2277,7 @@
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2330,7 +2324,7 @@
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2377,7 +2371,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2483,7 +2477,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H42" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2530,7 +2524,7 @@
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="H43" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2628,7 +2622,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -2675,7 +2669,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="6" t="inlineStr">
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -3067,7 +3061,7 @@
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -3161,7 +3155,7 @@
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -3298,7 +3292,7 @@
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" s="7" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -3541,7 +3535,7 @@
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" s="6" t="inlineStr">
+      <c r="H64" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -3588,7 +3582,7 @@
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="6" t="inlineStr">
+      <c r="H65" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -3737,7 +3731,7 @@
         </is>
       </c>
       <c r="G68" t="inlineStr"/>
-      <c r="H68" s="6" t="inlineStr">
+      <c r="H68" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -3784,7 +3778,7 @@
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="6" t="inlineStr">
+      <c r="H69" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -3839,7 +3833,7 @@
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="6" t="inlineStr">
+      <c r="H70" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -3937,22 +3931,22 @@
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I72" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>04_bert_transformers/245_Casillo2025_BeyondDomainDependencySecurity.pdf</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L72" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -4176,22 +4170,22 @@
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I77" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>04_bert_transformers/253_Ali2025_CloudBasedMachineLearning.pdf</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L77" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -4278,7 +4272,7 @@
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
-      <c r="H79" s="6" t="inlineStr">
+      <c r="H79" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -4372,7 +4366,7 @@
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="6" t="inlineStr">
+      <c r="H81" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -4423,7 +4417,7 @@
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
-      <c r="H82" s="6" t="inlineStr">
+      <c r="H82" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -4764,7 +4758,7 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="6" t="inlineStr">
+      <c r="H89" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -5007,22 +5001,22 @@
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I94" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr">
         <is>
           <t>05_llm/285_Alsanoosy2025_LargeLanguageModelRequirements.pdf</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L94" t="inlineStr">
         <is>
           <t>LLM</t>
@@ -5168,7 +5162,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H97" s="7" t="inlineStr">
+      <c r="H97" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -5364,7 +5358,7 @@
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="6" t="inlineStr">
+      <c r="H101" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -5411,7 +5405,7 @@
         </is>
       </c>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" s="6" t="inlineStr">
+      <c r="H102" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -5956,7 +5950,7 @@
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" s="6" t="inlineStr">
+      <c r="H113" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -6007,7 +6001,7 @@
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr"/>
-      <c r="H114" s="6" t="inlineStr">
+      <c r="H114" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -6105,7 +6099,7 @@
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr"/>
-      <c r="H116" s="6" t="inlineStr">
+      <c r="H116" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -6152,22 +6146,22 @@
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr"/>
-      <c r="H117" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I117" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr">
         <is>
-          <t>04_bert_transformers/349_Petrillo2026_ExplainableMethodSecurityRequirements.pdf</t>
-        </is>
-      </c>
-      <c r="K117" t="inlineStr"/>
+          <t>05_llm/349_Petrillo2026_ExplainableMethodSecurityRequirements.pdf</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L117" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -6391,7 +6385,7 @@
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="6" t="inlineStr">
+      <c r="H122" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -6532,7 +6526,7 @@
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr"/>
-      <c r="H125" s="6" t="inlineStr">
+      <c r="H125" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -6579,22 +6573,22 @@
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr"/>
-      <c r="H126" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I126" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr">
         <is>
           <t>04_bert_transformers/380_Nguyen2026_EvaluatingRobustnessHierarchicalMulti.pdf</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L126" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -6630,7 +6624,7 @@
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="6" t="inlineStr">
+      <c r="H127" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -6881,22 +6875,22 @@
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr"/>
-      <c r="H132" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I132" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr">
         <is>
           <t>03_aumentacion/400_Kaur2026_HybridApproachMultilevelMulti.pdf</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L132" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -6932,7 +6926,7 @@
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="6" t="inlineStr">
+      <c r="H133" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -6983,7 +6977,7 @@
         </is>
       </c>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="6" t="inlineStr">
+      <c r="H134" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -7034,7 +7028,7 @@
         </is>
       </c>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="6" t="inlineStr">
+      <c r="H135" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -7187,7 +7181,7 @@
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="6" t="inlineStr">
+      <c r="H138" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -7336,22 +7330,22 @@
       </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="I141" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H141" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr">
         <is>
           <t>04_bert_transformers/419_Rahman2026_RequibertTransferLearningSoftware.pdf</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L141" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -7434,7 +7428,7 @@
         </is>
       </c>
       <c r="G143" t="inlineStr"/>
-      <c r="H143" s="6" t="inlineStr">
+      <c r="H143" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -7481,7 +7475,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H144" s="6" t="inlineStr">
+      <c r="H144" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -7540,7 +7534,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H145" s="6" t="inlineStr">
+      <c r="H145" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -7614,119 +7608,108 @@
   <autoFilter ref="A1:M146"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I113" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I117" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I119" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I121" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I122" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I123" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I125" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I126" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I127" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I132" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I134" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I135" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I138" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I139" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I141" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I142" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I143" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I144" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I145" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I113" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I119" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I121" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I122" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I123" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I125" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I127" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I134" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I135" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I138" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I139" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I142" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I143" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I144" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I145" r:id="rId103"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7790,9 +7773,9 @@
         <v>35</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
+        <v>9</v>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>TITLE-ABS-KEY ( ( ( "non-functional" OR "non functional" OR nonfunctional OR quality OR NFR OR NFRs ) W/3 requirement* ) OR "software requirement*" OR "requirements specification*" OR "requirement* classification" OR "PROMISE NFR" OR "PROMISE_exp" ) AND TITLE-ABS-KEY ( classif* OR categori* ) AND TITLE-ABS-KEY ( "data augmentation" OR "text augmentation" OR "easy data augmentation" OR TextAttack OR TAOS OR "synthetic data" OR "synthetic sample*" OR oversampl* OR "over-sampling" OR resampl* OR SMOTE OR Tomek OR "class imbalance" OR "imbalanced data*" OR "imbalanced class*" OR "minority class*" OR "back translation" OR paraphras* ) AND PUBYEAR &gt; 2016 AND PUBYEAR &lt; 2027 AND ( LIMIT-TO ( DOCTYPE,"ar" ) OR LIMIT-TO ( DOCTYPE,"cp" ) OR LIMIT-TO ( DOCTYPE,"re" ) OR LIMIT-TO ( DOCTYPE,"ch" ) ) AND ( LIMIT-TO ( LANGUAGE,"English" ) OR LIMIT-TO ( LANGUAGE,"Spanish" ) )</t>
         </is>
@@ -7813,9 +7796,9 @@
         <v>95</v>
       </c>
       <c r="D3" t="n">
-        <v>16</v>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
+        <v>26</v>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>TITLE-ABS-KEY ( ( ( "non-functional" OR "non functional" OR nonfunctional OR quality OR NFR OR NFRs ) W/3 requirement* ) OR "software requirement*" OR "requirements specification*" OR "requirement* classification" OR "PROMISE NFR" OR "PROMISE_exp" ) AND TITLE-ABS-KEY ( classif* OR categori* ) AND TITLE-ABS-KEY ( BERT OR RoBERTa OR DistilBERT OR NoRBERT OR transformer* OR "pre-trained language model*" OR "pretrained language model*" OR "transfer learning" OR "fine tun*" ) AND PUBYEAR &gt; 2016 AND PUBYEAR &lt; 2027 AND ( LIMIT-TO ( DOCTYPE,"ar" ) OR LIMIT-TO ( DOCTYPE,"cp" ) OR LIMIT-TO ( DOCTYPE,"re" ) OR LIMIT-TO ( DOCTYPE,"ch" ) ) AND ( LIMIT-TO ( LANGUAGE,"English" ) OR LIMIT-TO ( LANGUAGE,"Spanish" ) )</t>
         </is>
@@ -7836,9 +7819,9 @@
         <v>59</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
+        <v>17</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>TITLE-ABS-KEY ( ( ( "non-functional" OR "non functional" OR nonfunctional OR quality OR NFR OR NFRs ) W/3 requirement* ) OR "software requirement*" OR "requirements specification*" OR "requirement* classification" OR "PROMISE NFR" OR "PROMISE_exp" ) AND TITLE-ABS-KEY ( classif* OR categori* ) AND TITLE-ABS-KEY ( "large language model*" OR LLM OR LLMs OR GPT* OR ChatGPT OR "generative AI" OR Llama OR Gemma OR Mistral OR Claude OR "zero-shot" OR "few-shot" OR "in-context learning" OR prompt* ) AND PUBYEAR &gt; 2016 AND PUBYEAR &lt; 2027 AND ( LIMIT-TO ( DOCTYPE,"ar" ) OR LIMIT-TO ( DOCTYPE,"cp" ) OR LIMIT-TO ( DOCTYPE,"re" ) OR LIMIT-TO ( DOCTYPE,"ch" ) ) AND ( LIMIT-TO ( LANGUAGE,"English" ) OR LIMIT-TO ( LANGUAGE,"Spanish" ) )</t>
         </is>
@@ -7859,9 +7842,9 @@
         <v>23</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
+        <v>6</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>TITLE-ABS-KEY ( ( ( "non-functional" OR "non functional" OR nonfunctional OR quality OR NFR OR NFRs ) W/3 requirement* ) OR "software requirement*" OR "requirements specification*" OR "requirement* classification" OR "PROMISE NFR" OR "PROMISE_exp" ) AND TITLE-ABS-KEY ( classif* OR categori* ) AND TITLE-ABS-KEY ( GitHub OR "issue tracker*" OR "issue report*" OR "open source" OR "open-source" OR "semi-supervised" OR "self-training" OR "pseudo-label*" OR "active learning" OR "weak supervision" OR "dataset construction" OR "gold standard" ) AND PUBYEAR &gt; 2016 AND PUBYEAR &lt; 2027 AND ( LIMIT-TO ( DOCTYPE,"ar" ) OR LIMIT-TO ( DOCTYPE,"cp" ) OR LIMIT-TO ( DOCTYPE,"re" ) OR LIMIT-TO ( DOCTYPE,"ch" ) ) AND ( LIMIT-TO ( LANGUAGE,"English" ) OR LIMIT-TO ( LANGUAGE,"Spanish" ) )</t>
         </is>
@@ -7966,16 +7949,12 @@
           <t>Automatically classifying user requests in crowdsourcing requirements engineering</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8162,7 +8141,7 @@
           <t>Software Requirements Classification using Deep-learning Approach with Various Hidden Layers</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8214,7 +8193,7 @@
           <t>Towards a FAIR Dataset for non-functional requirements</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8242,7 +8221,7 @@
           <t>EnsCL-CatBoost: A Strategic Framework for Software Requirements Classification</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8326,7 +8305,7 @@
           <t>Automated Classification and Identification of Non-Functional Requirements in Agile-Based Requirements Using Pre-Trained Language Models</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8354,7 +8333,7 @@
           <t>BET-BiLSTM Model: A Robust Solution for Automated Requirements Classification</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8462,7 +8441,7 @@
           <t>Enhancing Software Sustainability: Leveraging Large Language Models to Evaluate Security Requirements Fulfillment in Requirements Engineering</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8670,7 +8649,7 @@
           <t>Adaptive Data Augmentation Techniques for Software Requirements Classification Using Deep Learning</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8698,7 +8677,7 @@
           <t>An Intelligent Model to Predict Functional and Non-Functional Requirements From Software Requirements Specification</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8750,16 +8729,12 @@
           <t>Hybrid approach for multilevel multi-class requirement classification: Impact of stop-word removal and data augmentation</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8778,7 +8753,7 @@
           <t>Improving the Multi-Class Classification of Non-Functional Requirements in Spanish: A Study of Dataset Balancing and Performance</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8806,7 +8781,7 @@
           <t>On-demand generation of high-quality software engineering datasets using large language models and ontologies</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -8862,7 +8837,7 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9054,7 +9029,7 @@
           <t>A Zero-Shot Learning Approach to Classifying Requirements: A Preliminary Study</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9106,16 +9081,12 @@
           <t>Automatically classifying non-functional requirements using deep neural network</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9134,16 +9105,12 @@
           <t>BERT-CNN: Improving BERT for Requirements Classification using CNN</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -9162,7 +9129,7 @@
           <t>PRCBERT: Prompt Learning for Requirement Classification using BERT-based Pretrained Language Models</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9218,7 +9185,7 @@
           <t>An empirical study of automated privacy requirements classification in issue reports</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9246,7 +9213,7 @@
           <t>Comparing general purpose pre-trained Word and Sentence embeddings for Requirements Classification</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -9274,7 +9241,7 @@
           <t>Developing an Advanced Software Requirements Classification Model Using BERT: An Empirical Evaluation Study on Newly Generated Turkish Data</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9302,16 +9269,12 @@
           <t>Improving BERT model for requirements classification by bidirectional LSTM-CNN deep model</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9386,7 +9349,7 @@
           <t>Non Functional Requirements Identification and Classification Using Transfer Learning Model</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9414,7 +9377,7 @@
           <t>Requirements Classification Using FastText and BETO in Spanish Documents</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9466,7 +9429,7 @@
           <t>aeroBERT-Classifier: Classification of Aerospace Requirements Using BERT</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9494,7 +9457,7 @@
           <t>Classifying software security requirements into confidentiality, integrity, and availability using machine learning approaches</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9550,7 +9513,7 @@
           <t>Enhancing Software Requirements Classification with Semisupervised GAN-BERT Technique</t>
         </is>
       </c>
-      <c r="E61" s="6" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9706,7 +9669,7 @@
           <t>SSMBERT: A Space Science Mission Requirement Classification Method Based on BERT</t>
         </is>
       </c>
-      <c r="E67" s="6" t="inlineStr">
+      <c r="E67" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9790,7 +9753,7 @@
           <t>An approach to identifying functional and non-functional requirements in IT-project management using deep learning models</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr">
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -9842,7 +9805,7 @@
           <t>Automated Classification and Identification of Non-Functional Requirements in Agile-Based Requirements Using Pre-Trained Language Models</t>
         </is>
       </c>
-      <c r="E72" s="6" t="inlineStr">
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9870,7 +9833,7 @@
           <t>Automated NLP-Based Classification of Nonfunctional Requirements in Blockchain and Cross-Domain Software Systems Using BERT and Machine Learning</t>
         </is>
       </c>
-      <c r="E73" s="6" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9950,7 +9913,7 @@
           <t>BERT Fine-Tuning for Software Requirement Classification: Impact of Model Components and Dataset Size</t>
         </is>
       </c>
-      <c r="E76" s="6" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -9978,7 +9941,7 @@
           <t>BET-BiLSTM Model: A Robust Solution for Automated Requirements Classification</t>
         </is>
       </c>
-      <c r="E77" s="6" t="inlineStr">
+      <c r="E77" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10034,16 +9997,12 @@
           <t>Beyond domain dependency in security requirements identification</t>
         </is>
       </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F79" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10086,16 +10045,12 @@
           <t>Cloud-based machine learning for scalable classification of software requirements: Insights from the PROMISE dataset</t>
         </is>
       </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10142,7 +10097,7 @@
           <t>Enhancing Software Sustainability: Leveraging Large Language Models to Evaluate Security Requirements Fulfillment in Requirements Engineering</t>
         </is>
       </c>
-      <c r="E83" s="6" t="inlineStr">
+      <c r="E83" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10198,7 +10153,7 @@
           <t>Evaluating NLP Tools for AI in Software Requirements Analysis</t>
         </is>
       </c>
-      <c r="E85" s="6" t="inlineStr">
+      <c r="E85" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10226,7 +10181,7 @@
           <t>Explainable Security Requirements Classification Through Transformer Models</t>
         </is>
       </c>
-      <c r="E86" s="6" t="inlineStr">
+      <c r="E86" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10410,16 +10365,12 @@
           <t>Large Language Model for Requirements Classification: An Ensemble Approach</t>
         </is>
       </c>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F93" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10494,7 +10445,7 @@
           <t>Low-Level Hardware Requirement Classification Using Large Language Models: Challenges, Insights, and Future Directions for Embedded Control Systems</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr">
+      <c r="E96" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -10602,7 +10553,7 @@
           <t>On the Effectiveness of Zero-Shot and Few-Shot Pretrained Language Models for Software Requirement Classification</t>
         </is>
       </c>
-      <c r="E100" s="6" t="inlineStr">
+      <c r="E100" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10822,7 +10773,7 @@
           <t>A knowledge-driven semantic framework for non-functional requirement engineering in intelligent healthcare systems</t>
         </is>
       </c>
-      <c r="E108" s="6" t="inlineStr">
+      <c r="E108" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10850,7 +10801,7 @@
           <t>Adaptive Data Augmentation Techniques for Software Requirements Classification Using Deep Learning</t>
         </is>
       </c>
-      <c r="E109" s="6" t="inlineStr">
+      <c r="E109" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10878,7 +10829,7 @@
           <t>An Intelligent Model to Predict Functional and Non-Functional Requirements From Software Requirements Specification</t>
         </is>
       </c>
-      <c r="E110" s="6" t="inlineStr">
+      <c r="E110" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -10906,16 +10857,12 @@
           <t>An explainable method for security requirements classification through transformer models</t>
         </is>
       </c>
-      <c r="E111" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F111" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -11018,7 +10965,7 @@
           <t>Context-Aware Non-Functional Requirement Classification Using Functional Requirement Guidance and Domain-Specialized Representations</t>
         </is>
       </c>
-      <c r="E115" s="6" t="inlineStr">
+      <c r="E115" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11098,7 +11045,7 @@
           <t>ERC4AI: A BERT-Based Model for Ethical Requirements Classification in AI Systems</t>
         </is>
       </c>
-      <c r="E118" s="6" t="inlineStr">
+      <c r="E118" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11126,16 +11073,12 @@
           <t>Evaluating robustness of hierarchical and multi-label requirements classification: Effects of data partitioning and supervision design</t>
         </is>
       </c>
-      <c r="E119" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F119" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -11154,7 +11097,7 @@
           <t>EviReqRAG: An Evidence-Based Retrieval-Augmented Generation Framework for Software Requirements and Security Classification</t>
         </is>
       </c>
-      <c r="E120" s="6" t="inlineStr">
+      <c r="E120" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11234,16 +11177,12 @@
           <t>Hybrid approach for multilevel multi-class requirement classification: Impact of stop-word removal and data augmentation</t>
         </is>
       </c>
-      <c r="E123" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F123" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -11262,7 +11201,7 @@
           <t>Implicit security requirements classification with large language models using the OWASP application security verification standard: a shift-left approach</t>
         </is>
       </c>
-      <c r="E124" s="6" t="inlineStr">
+      <c r="E124" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11290,7 +11229,7 @@
           <t>KD-BERT: A Knowledge-Driven BERT Framework for Few-Shot Requirement Classification and Kano-Based Prioritization</t>
         </is>
       </c>
-      <c r="E125" s="6" t="inlineStr">
+      <c r="E125" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11374,16 +11313,12 @@
           <t>RequiBERT: Transfer learning for software requirements classifications</t>
         </is>
       </c>
-      <c r="E128" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F128" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -11430,7 +11365,7 @@
           <t>Requirements Classification Using Fine-Tuned Transformer Models: A Comparative Study of BERT, RoBERTa, and GPT-4o</t>
         </is>
       </c>
-      <c r="E130" s="6" t="inlineStr">
+      <c r="E130" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11458,7 +11393,7 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E131" s="6" t="inlineStr">
+      <c r="E131" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11486,7 +11421,7 @@
           <t>A Zero-Shot Learning Approach to Classifying Requirements: A Preliminary Study</t>
         </is>
       </c>
-      <c r="E132" s="6" t="inlineStr">
+      <c r="E132" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11514,7 +11449,7 @@
           <t>PRCBERT: Prompt Learning for Requirement Classification using BERT-based Pretrained Language Models</t>
         </is>
       </c>
-      <c r="E133" s="6" t="inlineStr">
+      <c r="E133" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11542,7 +11477,7 @@
           <t>Comparing general purpose pre-trained Word and Sentence embeddings for Requirements Classification</t>
         </is>
       </c>
-      <c r="E134" s="7" t="inlineStr">
+      <c r="E134" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -11594,7 +11529,7 @@
           <t>aeroBERT-Classifier: Classification of Aerospace Requirements Using BERT</t>
         </is>
       </c>
-      <c r="E136" s="6" t="inlineStr">
+      <c r="E136" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11726,7 +11661,7 @@
           <t>SSMBERT: A Space Science Mission Requirement Classification Method Based on BERT</t>
         </is>
       </c>
-      <c r="E141" s="6" t="inlineStr">
+      <c r="E141" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11782,7 +11717,7 @@
           <t>Which AI Technique Is Better to Classify Requirements? An Experiment with SVM, LSTM, and ChatGPT</t>
         </is>
       </c>
-      <c r="E143" s="7" t="inlineStr">
+      <c r="E143" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -11910,7 +11845,7 @@
           <t>Automating Requirements Classification: A Systematic Literature Review and Ensemble LLM-Based Approach</t>
         </is>
       </c>
-      <c r="E148" s="6" t="inlineStr">
+      <c r="E148" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -11938,7 +11873,7 @@
           <t>BET-BiLSTM Model: A Robust Solution for Automated Requirements Classification</t>
         </is>
       </c>
-      <c r="E149" s="6" t="inlineStr">
+      <c r="E149" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12018,7 +11953,7 @@
           <t>Enhancing Software Sustainability: Leveraging Large Language Models to Evaluate Security Requirements Fulfillment in Requirements Engineering</t>
         </is>
       </c>
-      <c r="E152" s="6" t="inlineStr">
+      <c r="E152" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12046,7 +11981,7 @@
           <t>Explainable Security Requirements Classification Through Transformer Models</t>
         </is>
       </c>
-      <c r="E153" s="6" t="inlineStr">
+      <c r="E153" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12202,7 +12137,7 @@
           <t>How Reliable Are GPT-4o and LLAMA3.3-70B in Classifying Natural Language Requirements?: The Impact of the Temperature Setting</t>
         </is>
       </c>
-      <c r="E159" s="6" t="inlineStr">
+      <c r="E159" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12254,16 +12189,12 @@
           <t>Large Language Model for Requirements Classification: An Ensemble Approach</t>
         </is>
       </c>
-      <c r="E161" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F161" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -12338,7 +12269,7 @@
           <t>Low-Level Hardware Requirement Classification Using Large Language Models: Challenges, Insights, and Future Directions for Embedded Control Systems</t>
         </is>
       </c>
-      <c r="E164" s="7" t="inlineStr">
+      <c r="E164" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -12394,7 +12325,7 @@
           <t>On the Effectiveness of Zero-Shot and Few-Shot Pretrained Language Models for Software Requirement Classification</t>
         </is>
       </c>
-      <c r="E166" s="6" t="inlineStr">
+      <c r="E166" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12422,7 +12353,7 @@
           <t>One Size Does Not Fit All: On the Role of Batch Size in Classifying Requirements with LLMs</t>
         </is>
       </c>
-      <c r="E167" s="6" t="inlineStr">
+      <c r="E167" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12722,7 +12653,7 @@
           <t>EviReqRAG: An Evidence-Based Retrieval-Augmented Generation Framework for Software Requirements and Security Classification</t>
         </is>
       </c>
-      <c r="E178" s="6" t="inlineStr">
+      <c r="E178" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12802,7 +12733,7 @@
           <t>Implicit security requirements classification with large language models using the OWASP application security verification standard: a shift-left approach</t>
         </is>
       </c>
-      <c r="E181" s="6" t="inlineStr">
+      <c r="E181" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12830,7 +12761,7 @@
           <t>Improving the Multi-Class Classification of Non-Functional Requirements in Spanish: A Study of Dataset Balancing and Performance</t>
         </is>
       </c>
-      <c r="E182" s="6" t="inlineStr">
+      <c r="E182" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12858,7 +12789,7 @@
           <t>KD-BERT: A Knowledge-Driven BERT Framework for Few-Shot Requirement Classification and Kano-Based Prioritization</t>
         </is>
       </c>
-      <c r="E183" s="6" t="inlineStr">
+      <c r="E183" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12914,7 +12845,7 @@
           <t>On-demand generation of high-quality software engineering datasets using large language models and ontologies</t>
         </is>
       </c>
-      <c r="E185" s="6" t="inlineStr">
+      <c r="E185" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -12994,7 +12925,7 @@
           <t>Requirements Classification Using Fine-Tuned Transformer Models: A Comparative Study of BERT, RoBERTa, and GPT-4o</t>
         </is>
       </c>
-      <c r="E188" s="6" t="inlineStr">
+      <c r="E188" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13022,7 +12953,7 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E189" s="6" t="inlineStr">
+      <c r="E189" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13098,16 +13029,12 @@
           <t>Automatically classifying user requests in crowdsourcing requirements engineering</t>
         </is>
       </c>
-      <c r="E192" s="5" t="inlineStr">
-        <is>
-          <t>ScienceDirect (UPeU)</t>
-        </is>
-      </c>
-      <c r="F192" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13314,7 +13241,7 @@
           <t>A Novel Hybrid Deep Learning Model for Detecting and Classifying Non-Functional Requirements of Mobile Apps Issues</t>
         </is>
       </c>
-      <c r="E200" s="6" t="inlineStr">
+      <c r="E200" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13342,7 +13269,7 @@
           <t>An empirical study of automated privacy requirements classification in issue reports</t>
         </is>
       </c>
-      <c r="E201" s="6" t="inlineStr">
+      <c r="E201" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13370,7 +13297,7 @@
           <t>aeroBERT-Classifier: Classification of Aerospace Requirements Using BERT</t>
         </is>
       </c>
-      <c r="E202" s="6" t="inlineStr">
+      <c r="E202" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13398,7 +13325,7 @@
           <t>Enhancing Software Requirements Classification with Semisupervised GAN-BERT Technique</t>
         </is>
       </c>
-      <c r="E203" s="6" t="inlineStr">
+      <c r="E203" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13482,7 +13409,7 @@
           <t>Low-Level Hardware Requirement Classification Using Large Language Models: Challenges, Insights, and Future Directions for Embedded Control Systems</t>
         </is>
       </c>
-      <c r="E206" s="7" t="inlineStr">
+      <c r="E206" s="6" t="inlineStr">
         <is>
           <t>Sin DOI (buscar por título)</t>
         </is>
@@ -13642,7 +13569,7 @@
           <t>SeqFAL: A Federated Active Learning Framework for Private and Efficient Labeling of Security Requirements</t>
         </is>
       </c>
-      <c r="E212" s="6" t="inlineStr">
+      <c r="E212" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13670,7 +13597,7 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E213" s="6" t="inlineStr">
+      <c r="E213" s="5" t="inlineStr">
         <is>
           <t>Acceso abierto (navegador)</t>
         </is>
@@ -13685,173 +13612,159 @@
   <autoFilter ref="A1:F213"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F110" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F111" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F114" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F115" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F116" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F118" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F119" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F120" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F121" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F123" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F124" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F125" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F126" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F127" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F128" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F129" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F130" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F131" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F132" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F133" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F134" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F136" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F137" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F141" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F149" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F150" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F152" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F153" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F154" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F156" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F159" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F161" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F166" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F192" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F110" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F114" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F115" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F116" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F118" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F120" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F121" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F124" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F125" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F126" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F127" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F129" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F130" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F131" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F132" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F133" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F134" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F136" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F137" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F141" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F149" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F150" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F152" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F153" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F154" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F156" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F159" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F166" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId154"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
RSL: 25 textos completos más de acceso abierto (67 extraídos, 58 en la síntesis)
- descargar_abiertos.py: descarga con curl, rutas directas de IEEE y MDPI y
  verificación del título (con normalización de ligaduras)
- Lote 09: 25 estudios; 4 excluidos (CE1 aeroespaciales, CE2 trazabilidad y Kano)
- Hallazgos: dos estudios comparan varias aumentaciones (Petrillo 2025, Aldhafer 2026);
  SMOTE y SMOTE-Tomek antes de partir (Vijayvargiya, Abbas); el protocolo cambia
  el F1 macro de 0.97 a 0.80 (Almohammady)
- Tabla de síntesis dividida en dos partes; referencia GitReq duplicada eliminada

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Articulos/PDF/INDICE_ARTICULOS.xlsx
+++ b/Articulos/PDF/INDICE_ARTICULOS.xlsx
@@ -1803,22 +1803,22 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>03_aumentacion/89_Vijayvargiya2022_SoftwareRequirementsClassificationUsing.pdf</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>Aprendizaje profundo</t>
@@ -1897,22 +1897,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>06_ml_dl_clasico/97_Yahya2023_NovelHybridDeepLearning.pdf</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>Aprendizaje profundo</t>
@@ -1995,22 +1995,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
           <t>04_bert_transformers/100_Sangaroonsilp2023_EmpiricalStudyAutomatedPrivacy.pdf</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Excluido (CE2)</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -2089,22 +2089,22 @@
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>04_bert_transformers/112_Yucalar2023_DevelopingAdvancedSoftwareRequirements.pdf</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -2277,22 +2277,22 @@
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>04_bert_transformers/127_Khan2023_FunctionalRequirementsIdentificationClas.pdf</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -2477,22 +2477,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>04_bert_transformers/139_Tikayat2023_AerobertClassifierClassificationAerospac.pdf</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Excluido (CE1)</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -2524,22 +2524,22 @@
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>04_bert_transformers/156_Bagies2024_ClassifyingSoftwareSecurityRequirements.pdf</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -2669,22 +2669,22 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I46" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
           <t>03_aumentacion/164_Abbas2024_EnsclCatboostStrategicFramework.pdf</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>ML clásico</t>
@@ -3061,22 +3061,22 @@
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I54" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
           <t>04_bert_transformers/193_Zhu2024_SsmbertSpaceScienceMission.pdf</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Excluido (CE1)</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -3535,22 +3535,22 @@
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>01_semillas/231_Alhaizaey2025_AutomatedClassificationIdentificationFun.pdf</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -3778,22 +3778,22 @@
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>04_bert_transformers/241_Eltahier2025_BertFineTuningSoftware.pdf</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L69" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -4272,22 +4272,22 @@
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
-      <c r="H79" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I79" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
           <t>05_llm/261_Subahi2025_EnhancingSoftwareSustainabilityLeveragin.pdf</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L79" t="inlineStr">
         <is>
           <t>LLM</t>
@@ -4417,22 +4417,22 @@
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
-      <c r="H82" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I82" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>03_aumentacion/267_Petrillo2025_ExplainableSecurityRequirementsClassific.pdf</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L82" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -4758,22 +4758,22 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I89" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
           <t>05_llm/275_Karlsson2025_ReliableLlama3ClassifyingNatural.pdf</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L89" t="inlineStr">
         <is>
           <t>LLM</t>
@@ -5358,22 +5358,22 @@
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I101" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr">
         <is>
           <t>05_llm/299_Shafikuzzaman2025_EffectivenessZeroShotShot.pdf</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L101" t="inlineStr">
         <is>
           <t>LLM</t>
@@ -5950,22 +5950,22 @@
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I113" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H113" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>04_bert_transformers/336_Bhar2026_KnowledgeDrivenSemanticFramework.pdf</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L113" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -6001,22 +6001,22 @@
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr"/>
-      <c r="H114" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I114" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H114" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr">
         <is>
           <t>03_aumentacion/344_Aldhafer2026_AdaptiveDataAugmentationTechniques.pdf</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L114" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -6099,22 +6099,22 @@
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr"/>
-      <c r="H116" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I116" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H116" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>04_bert_transformers/348_Said2026_IntelligentModelPredictFunctional.pdf</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L116" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -6385,22 +6385,22 @@
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I122" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr">
         <is>
           <t>04_bert_transformers/363_Almohammady2026_ContextAwareFunctionalRequirement.pdf</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L122" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -6624,22 +6624,22 @@
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I127" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr">
         <is>
           <t>05_llm/381_Aloufi2026_EvireqragEvidenceBasedRetrieval.pdf</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L127" t="inlineStr">
         <is>
           <t>LLM</t>
@@ -6977,22 +6977,22 @@
         </is>
       </c>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I134" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr">
         <is>
           <t>03_aumentacion/403_LimayllaLunarejo2026_ImprovingMultiClassClassification.pdf</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L134" t="inlineStr">
         <is>
           <t>ML clásico</t>
@@ -7028,22 +7028,22 @@
         </is>
       </c>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I135" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr">
         <is>
           <t>04_bert_transformers/407_Almoqren2026_BertKnowledgeDrivenBert.pdf</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Excluido (CE2)</t>
+        </is>
+      </c>
       <c r="L135" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -7181,22 +7181,22 @@
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I138" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H138" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr">
         <is>
           <t>03_aumentacion/414_Bishop2026_DemandGenerationHighQuality.pdf</t>
         </is>
       </c>
-      <c r="K138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L138" t="inlineStr">
         <is>
           <t>LLM</t>
@@ -7475,22 +7475,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H144" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I144" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H144" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr">
         <is>
           <t>06_ml_dl_clasico/425_Alhoshan2026_SeqfalFederatedActiveLearning.pdf</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L144" t="inlineStr">
         <is>
           <t>ML clásico</t>
@@ -7534,22 +7534,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H145" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="I145" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="H145" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr">
         <is>
           <t>04_bert_transformers/430_Bagies2026_TransformerBasedClassificationSecurity.pdf</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="L145" t="inlineStr">
         <is>
           <t>Transformer</t>
@@ -7625,91 +7625,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I113" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I119" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I121" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I122" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I123" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I125" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I127" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I134" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I135" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I138" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I139" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I142" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I143" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I144" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I145" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I119" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I121" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I123" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I125" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I139" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I142" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I143" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7773,7 +7748,7 @@
         <v>35</v>
       </c>
       <c r="D2" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
@@ -7796,7 +7771,7 @@
         <v>95</v>
       </c>
       <c r="D3" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
@@ -7819,7 +7794,7 @@
         <v>59</v>
       </c>
       <c r="D4" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7842,7 +7817,7 @@
         <v>23</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -8141,16 +8116,12 @@
           <t>Software Requirements Classification using Deep-learning Approach with Various Hidden Layers</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8221,16 +8192,12 @@
           <t>EnsCL-CatBoost: A Strategic Framework for Software Requirements Classification</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8305,16 +8272,12 @@
           <t>Automated Classification and Identification of Non-Functional Requirements in Agile-Based Requirements Using Pre-Trained Language Models</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8441,16 +8404,12 @@
           <t>Enhancing Software Sustainability: Leveraging Large Language Models to Evaluate Security Requirements Fulfillment in Requirements Engineering</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8649,16 +8608,12 @@
           <t>Adaptive Data Augmentation Techniques for Software Requirements Classification Using Deep Learning</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8677,16 +8632,12 @@
           <t>An Intelligent Model to Predict Functional and Non-Functional Requirements From Software Requirements Specification</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8753,16 +8704,12 @@
           <t>Improving the Multi-Class Classification of Non-Functional Requirements in Spanish: A Study of Dataset Balancing and Performance</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8781,16 +8728,12 @@
           <t>On-demand generation of high-quality software engineering datasets using large language models and ontologies</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8837,16 +8780,12 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9185,16 +9124,12 @@
           <t>An empirical study of automated privacy requirements classification in issue reports</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -9241,16 +9176,12 @@
           <t>Developing an Advanced Software Requirements Classification Model Using BERT: An Empirical Evaluation Study on Newly Generated Turkish Data</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9349,16 +9280,12 @@
           <t>Non Functional Requirements Identification and Classification Using Transfer Learning Model</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9429,16 +9356,12 @@
           <t>aeroBERT-Classifier: Classification of Aerospace Requirements Using BERT</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -9457,16 +9380,12 @@
           <t>Classifying software security requirements into confidentiality, integrity, and availability using machine learning approaches</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9669,16 +9588,12 @@
           <t>SSMBERT: A Space Science Mission Requirement Classification Method Based on BERT</t>
         </is>
       </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9805,16 +9720,12 @@
           <t>Automated Classification and Identification of Non-Functional Requirements in Agile-Based Requirements Using Pre-Trained Language Models</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9913,16 +9824,12 @@
           <t>BERT Fine-Tuning for Software Requirement Classification: Impact of Model Components and Dataset Size</t>
         </is>
       </c>
-      <c r="E76" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F76" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10097,16 +10004,12 @@
           <t>Enhancing Software Sustainability: Leveraging Large Language Models to Evaluate Security Requirements Fulfillment in Requirements Engineering</t>
         </is>
       </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -10181,16 +10084,12 @@
           <t>Explainable Security Requirements Classification Through Transformer Models</t>
         </is>
       </c>
-      <c r="E86" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F86" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10553,16 +10452,12 @@
           <t>On the Effectiveness of Zero-Shot and Few-Shot Pretrained Language Models for Software Requirement Classification</t>
         </is>
       </c>
-      <c r="E100" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F100" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10773,16 +10668,12 @@
           <t>A knowledge-driven semantic framework for non-functional requirement engineering in intelligent healthcare systems</t>
         </is>
       </c>
-      <c r="E108" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -10801,16 +10692,12 @@
           <t>Adaptive Data Augmentation Techniques for Software Requirements Classification Using Deep Learning</t>
         </is>
       </c>
-      <c r="E109" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -10829,16 +10716,12 @@
           <t>An Intelligent Model to Predict Functional and Non-Functional Requirements From Software Requirements Specification</t>
         </is>
       </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -10965,16 +10848,12 @@
           <t>Context-Aware Non-Functional Requirement Classification Using Functional Requirement Guidance and Domain-Specialized Representations</t>
         </is>
       </c>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -11097,16 +10976,12 @@
           <t>EviReqRAG: An Evidence-Based Retrieval-Augmented Generation Framework for Software Requirements and Security Classification</t>
         </is>
       </c>
-      <c r="E120" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F120" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -11229,16 +11104,12 @@
           <t>KD-BERT: A Knowledge-Driven BERT Framework for Few-Shot Requirement Classification and Kano-Based Prioritization</t>
         </is>
       </c>
-      <c r="E125" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F125" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -11393,16 +11264,12 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E131" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F131" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -11529,16 +11396,12 @@
           <t>aeroBERT-Classifier: Classification of Aerospace Requirements Using BERT</t>
         </is>
       </c>
-      <c r="E136" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F136" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -11661,16 +11524,12 @@
           <t>SSMBERT: A Space Science Mission Requirement Classification Method Based on BERT</t>
         </is>
       </c>
-      <c r="E141" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F141" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E141" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -11953,16 +11812,12 @@
           <t>Enhancing Software Sustainability: Leveraging Large Language Models to Evaluate Security Requirements Fulfillment in Requirements Engineering</t>
         </is>
       </c>
-      <c r="E152" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F152" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E152" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -11981,16 +11836,12 @@
           <t>Explainable Security Requirements Classification Through Transformer Models</t>
         </is>
       </c>
-      <c r="E153" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F153" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E153" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -12137,16 +11988,12 @@
           <t>How Reliable Are GPT-4o and LLAMA3.3-70B in Classifying Natural Language Requirements?: The Impact of the Temperature Setting</t>
         </is>
       </c>
-      <c r="E159" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F159" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E159" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -12325,16 +12172,12 @@
           <t>On the Effectiveness of Zero-Shot and Few-Shot Pretrained Language Models for Software Requirement Classification</t>
         </is>
       </c>
-      <c r="E166" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F166" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E166" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -12653,16 +12496,12 @@
           <t>EviReqRAG: An Evidence-Based Retrieval-Augmented Generation Framework for Software Requirements and Security Classification</t>
         </is>
       </c>
-      <c r="E178" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F178" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E178" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12761,16 +12600,12 @@
           <t>Improving the Multi-Class Classification of Non-Functional Requirements in Spanish: A Study of Dataset Balancing and Performance</t>
         </is>
       </c>
-      <c r="E182" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F182" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E182" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12789,16 +12624,12 @@
           <t>KD-BERT: A Knowledge-Driven BERT Framework for Few-Shot Requirement Classification and Kano-Based Prioritization</t>
         </is>
       </c>
-      <c r="E183" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F183" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E183" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -12845,16 +12676,12 @@
           <t>On-demand generation of high-quality software engineering datasets using large language models and ontologies</t>
         </is>
       </c>
-      <c r="E185" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F185" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -12953,16 +12780,12 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E189" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F189" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -13241,16 +13064,12 @@
           <t>A Novel Hybrid Deep Learning Model for Detecting and Classifying Non-Functional Requirements of Mobile Apps Issues</t>
         </is>
       </c>
-      <c r="E200" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F200" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E200" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -13269,16 +13088,12 @@
           <t>An empirical study of automated privacy requirements classification in issue reports</t>
         </is>
       </c>
-      <c r="E201" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F201" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -13297,16 +13112,12 @@
           <t>aeroBERT-Classifier: Classification of Aerospace Requirements Using BERT</t>
         </is>
       </c>
-      <c r="E202" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F202" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E202" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -13569,16 +13380,12 @@
           <t>SeqFAL: A Federated Active Learning Framework for Private and Efficient Labeling of Security Requirements</t>
         </is>
       </c>
-      <c r="E212" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F212" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E212" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -13597,16 +13404,12 @@
           <t>Transformer-Based Classification of Security-Related Mobile App Reviews Using Active Learning</t>
         </is>
       </c>
-      <c r="E213" s="5" t="inlineStr">
-        <is>
-          <t>Acceso abierto (navegador)</t>
-        </is>
-      </c>
-      <c r="F213" s="3" t="inlineStr">
-        <is>
-          <t>abrir</t>
-        </is>
-      </c>
+      <c r="E213" s="4" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F213"/>
@@ -13618,153 +13421,110 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F110" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F114" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F115" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F116" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F118" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F120" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F121" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F124" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F125" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F126" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F127" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F129" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F130" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F131" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F132" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F133" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F134" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F136" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F137" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F141" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F149" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F150" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F152" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F153" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F154" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F156" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F159" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F166" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F114" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F116" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F118" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F121" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F124" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F126" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F127" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F129" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F130" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F132" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F133" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F134" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F137" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F149" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F150" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F154" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F156" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId111"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>